<commit_message>
Saving to file is working. Whole process is working from end-to-end.
</commit_message>
<xml_diff>
--- a/SampleFiles/OutputFile.xlsx
+++ b/SampleFiles/OutputFile.xlsx
@@ -17,7 +17,46 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t>Hello World!</x:t>
+    <x:t>Sheet1 colunn 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet1 colunn 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet1 colunn 3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet1 colunn 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet1 colunn 5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet1 colunn 6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet2 colunn 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet2 colunn 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet2 colunn 3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet2 colunn 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet2 colunn 5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sheet2 colunn 6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>B17 Text</x:t>
+  </x:si>
+  <x:si>
+    <x:t>F16 Text</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -368,9 +407,81 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData/>
+  <x:sheetData>
+    <x:row r="1" spans="1:6">
+      <x:c r="A1" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
+      <x:c r="A2" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C2" s="0">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C3" s="0">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C4" s="0">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
@@ -384,12 +495,42 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:A2"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="2" spans="1:1">
-      <x:c r="A2" s="0" t="s">
-        <x:v>0</x:v>
+    <x:row r="1" spans="1:6">
+      <x:c r="A1" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
+      <x:c r="F2" s="0">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="F3" s="0">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="F4" s="0">
+        <x:v>10</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>